<commit_message>
Use python -m to run uvicorn and streamlit
Update startup instructions and in-app messages to recommend invoking uvicorn and Streamlit via `python -m` so the virtualenv-installed entrypoints are used. Changes: README and app/main.py docstring updated, client/streamlit_app.py error messages adjusted, removed stray Excel temp lock file (~$...) and updated the corpus .xlsx and .DS_Store binaries.
</commit_message>
<xml_diff>
--- a/corpus/rq1_accuracy_audit_populated.xlsx
+++ b/corpus/rq1_accuracy_audit_populated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rakelosksigurdardottir/Documents/IE University/Capstone/NARR/NARR_prototype/corpus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{114F85AA-2229-9C4F-9F88-375F58C30FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C87105B8-7AAD-B643-884F-420D5F8E0D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28080" windowHeight="18460" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28080" windowHeight="18460" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2913" uniqueCount="611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2919" uniqueCount="612">
   <si>
     <t>RQ1 Accuracy Audit — Scoring Sheet Instructions</t>
   </si>
@@ -1935,6 +1935,9 @@
   </si>
   <si>
     <t>all fabrications soft</t>
+  </si>
+  <si>
+    <t>  </t>
   </si>
 </sst>
 </file>
@@ -2049,7 +2052,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2076,7 +2079,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -2535,7 +2537,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:I338"/>
+  <dimension ref="A1:I342"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2688,7 +2690,7 @@
       </c>
       <c r="I5" s="5"/>
     </row>
-    <row r="6" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>33</v>
       </c>
@@ -3122,7 +3124,7 @@
       </c>
       <c r="I21" s="5"/>
     </row>
-    <row r="22" spans="1:9" ht="28" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>67</v>
       </c>
@@ -3230,7 +3232,7 @@
       </c>
       <c r="I25" s="5"/>
     </row>
-    <row r="26" spans="1:9" ht="28" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
         <v>67</v>
       </c>
@@ -3875,6 +3877,9 @@
       <c r="E50" s="11" t="s">
         <v>110</v>
       </c>
+      <c r="F50" t="s">
+        <v>101</v>
+      </c>
       <c r="G50" s="11" t="s">
         <v>104</v>
       </c>
@@ -4485,7 +4490,7 @@
       <c r="H73" t="s">
         <v>39</v>
       </c>
-      <c r="I73" s="14" t="s">
+      <c r="I73" t="s">
         <v>591</v>
       </c>
     </row>
@@ -4593,7 +4598,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:9" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>124</v>
       </c>
@@ -5310,7 +5315,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:9" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>180</v>
       </c>
@@ -5339,7 +5344,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="192" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:9" ht="192" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>180</v>
       </c>
@@ -5485,6 +5490,9 @@
       <c r="E111" s="11" t="s">
         <v>188</v>
       </c>
+      <c r="F111" t="s">
+        <v>98</v>
+      </c>
       <c r="G111" s="11" t="s">
         <v>176</v>
       </c>
@@ -5560,6 +5568,9 @@
       <c r="E114" s="11" t="s">
         <v>192</v>
       </c>
+      <c r="F114" t="s">
+        <v>98</v>
+      </c>
       <c r="G114" s="11" t="s">
         <v>157</v>
       </c>
@@ -5609,6 +5620,9 @@
       <c r="E116" s="11" t="s">
         <v>194</v>
       </c>
+      <c r="F116" t="s">
+        <v>98</v>
+      </c>
       <c r="G116" s="11" t="s">
         <v>157</v>
       </c>
@@ -5694,7 +5708,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="32" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>180</v>
       </c>
@@ -5908,7 +5922,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:9" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>206</v>
       </c>
@@ -6119,7 +6133,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="224" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:9" ht="224" hidden="1" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>206</v>
       </c>
@@ -6920,7 +6934,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="166" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>259</v>
       </c>
@@ -7544,7 +7558,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="190" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>289</v>
       </c>
@@ -7768,6 +7782,9 @@
       <c r="E198" s="11" t="s">
         <v>307</v>
       </c>
+      <c r="F198" t="s">
+        <v>37</v>
+      </c>
       <c r="G198" s="11" t="s">
         <v>584</v>
       </c>
@@ -11427,11 +11444,16 @@
         <v>39</v>
       </c>
     </row>
+    <row r="342" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="G342" s="11" t="s">
+        <v>611</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I338" xr:uid="{00000000-0009-0000-0000-000001000000}">
-    <filterColumn colId="7">
+    <filterColumn colId="5">
       <filters>
-        <filter val="Fabricated"/>
+        <filter val="Hedging"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -11442,7 +11464,7 @@
     <dataValidation type="list" allowBlank="1" sqref="C2:C7954" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"time_series,categorical,geospatial"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" error="Pick a claim type" prompt="Select claim type" sqref="F1:F1048576" xr:uid="{5C646DF3-58D2-6F41-9D7D-42A711A89663}">
+    <dataValidation type="list" allowBlank="1" error="Pick a claim type" prompt="Select claim type" sqref="F1:F342 F344:F1048576" xr:uid="{5C646DF3-58D2-6F41-9D7D-42A711A89663}">
       <formula1>"Numerical,Directional,Entity,Fabrication,Hedging, Interpretation, Data note"</formula1>
     </dataValidation>
   </dataValidations>
@@ -11609,7 +11631,7 @@
         <v>0.95238095238095233</v>
       </c>
       <c r="L3" s="5" t="str">
-        <f t="shared" ref="L3:L21" si="1">IF(J3=0,"Yes","No")</f>
+        <f t="shared" ref="L3:L19" si="1">IF(J3=0,"Yes","No")</f>
         <v>No</v>
       </c>
       <c r="M3" s="5" t="s">
@@ -11722,7 +11744,7 @@
       <c r="N5" s="5">
         <v>9.4600000000000009</v>
       </c>
-      <c r="O5" s="15" t="s">
+      <c r="O5" s="14" t="s">
         <v>591</v>
       </c>
     </row>
@@ -13989,7 +14011,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -14039,7 +14061,7 @@
       <c r="A5" s="9" t="s">
         <v>533</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="15">
         <f>COUNTIFS('Claim Audit'!$F:$F,"Numerical",'Claim Audit'!$H:$H,"Accurate")/COUNTIF('Claim Audit'!$F:$F,"Numerical")</f>
         <v>1</v>
       </c>
@@ -14049,7 +14071,7 @@
       <c r="A6" s="9" t="s">
         <v>534</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="15">
         <f>COUNTIFS('Claim Audit'!$F:$F,"Directional",'Claim Audit'!$H:$H,"Accurate")/COUNTIF('Claim Audit'!$F:$F,"Directional")</f>
         <v>1</v>
       </c>
@@ -14059,7 +14081,7 @@
       <c r="A7" s="9" t="s">
         <v>609</v>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="16">
         <f>COUNTIFS('Claim Audit'!$F:$F,"Interpretation",'Claim Audit'!$H:$H,"Accurate")/COUNTIF('Claim Audit'!$F:$F,"Interpretation")</f>
         <v>0.93023255813953487</v>
       </c>
@@ -14069,7 +14091,7 @@
       <c r="A8" s="9" t="s">
         <v>535</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15">
         <f>COUNTIFS('Claim Audit'!$F:$F,"Entity",'Claim Audit'!$H:$H,"Accurate")/COUNTIF('Claim Audit'!$F:$F,"Entity")</f>
         <v>1</v>
       </c>
@@ -14091,7 +14113,7 @@
       <c r="A10" s="9" t="s">
         <v>537</v>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="16">
         <f>COUNTIF('Claim Audit'!H:H,"Accurate")/B4</f>
         <v>0.98219584569732943</v>
       </c>
@@ -14101,7 +14123,7 @@
       <c r="A11" s="9" t="s">
         <v>538</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="15">
         <f>COUNTIFS('Claim Audit'!F:F,"Hedging",'Claim Audit'!H:H,"Accurate")/COUNTIF('Claim Audit'!F:F,"Hedging")</f>
         <v>1</v>
       </c>
@@ -14250,7 +14272,7 @@
       <c r="A28" s="9" t="s">
         <v>606</v>
       </c>
-      <c r="B28" s="17">
+      <c r="B28" s="16">
         <f>12/16</f>
         <v>0.75</v>
       </c>
@@ -14260,11 +14282,17 @@
       <c r="A29" s="9" t="s">
         <v>607</v>
       </c>
-      <c r="B29" s="16">
+      <c r="B29" s="15">
         <f xml:space="preserve"> 16/16</f>
         <v>1</v>
       </c>
       <c r="C29" s="10"/>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B33">
+        <f>COUNTIF('Claim Audit'!$F:$F, "Directional")</f>
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>